<commit_message>
More on OL accurals mapping and excel files
</commit_message>
<xml_diff>
--- a/data/obx_xlsx/BAKKA.OL.xlsx
+++ b/data/obx_xlsx/BAKKA.OL.xlsx
@@ -9629,7 +9629,10 @@
       <c r="Q47" s="16">
         <v>372.52</v>
       </c>
-      <c r="R47" s="15"/>
+      <c r="R47" s="15">
+        <f>SUM(R48:R56,R64)</f>
+        <v>257.52</v>
+      </c>
       <c r="S47" s="16">
         <v>184.13</v>
       </c>

</xml_diff>